<commit_message>
feat: add Google OAuth, email verification, pricing page, and 3D sphere
- Google OAuth login/register flow with callback and welcome pages
- Email verification with resend support via Resend API
- Prisma migrations for OAuth user and email verification fields
- Mail service using Resend for transactional emails
- Pricing page UI component
- 3D product sphere canvas with winner overlay and prize tier stack
- Updated auth views (login, register) with new flows
- Site header updates and i18n message additions

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/product/LichSuGiai.xlsx
+++ b/product/LichSuGiai.xlsx
@@ -375,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:C6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -413,149 +413,9 @@
         <v>Giải ba</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>777928125</v>
-      </c>
-      <c r="B7" t="str">
-        <v>NGUYỄN HOÀNG ANH KIỆT</v>
-      </c>
-      <c r="C7" t="str">
-        <v>777928125</v>
-      </c>
-      <c r="D7" t="str">
-        <v>../img/KhachMoi/KhongAnh.jpg</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>779287899</v>
-      </c>
-      <c r="B8" t="str">
-        <v>TRẦN BÌNH DƯƠNG</v>
-      </c>
-      <c r="C8" t="str">
-        <v>779287899</v>
-      </c>
-      <c r="D8" t="str">
-        <v>../img/KhachMoi/KhongAnh.jpg</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>779432408</v>
-      </c>
-      <c r="B9" t="str">
-        <v>BÙI PHƯƠNG UYÊN</v>
-      </c>
-      <c r="C9" t="str">
-        <v>779432408</v>
-      </c>
-      <c r="D9" t="str">
-        <v>../img/KhachMoi/KhongAnh.jpg</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>777969668</v>
-      </c>
-      <c r="B10" t="str">
-        <v>VŨ HOÀI AN</v>
-      </c>
-      <c r="C10" t="str">
-        <v>777969668</v>
-      </c>
-      <c r="D10" t="str">
-        <v>../img/KhachMoi/KhongAnh.jpg</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>777194829</v>
-      </c>
-      <c r="B11" t="str">
-        <v>TRẦN BÁ TIẾN</v>
-      </c>
-      <c r="C11" t="str">
-        <v>777194829</v>
-      </c>
-      <c r="D11" t="str">
-        <v>../img/KhachMoi/KhongAnh.jpg</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>779025768</v>
-      </c>
-      <c r="B12" t="str">
-        <v>PHẠM THỊ LY</v>
-      </c>
-      <c r="C12" t="str">
-        <v>779025768</v>
-      </c>
-      <c r="D12" t="str">
-        <v>../img/KhachMoi/KhongAnh.jpg</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>776932381</v>
-      </c>
-      <c r="B13" t="str">
-        <v>VŨ ĐÌNH PHÚC</v>
-      </c>
-      <c r="C13" t="str">
-        <v>776932381</v>
-      </c>
-      <c r="D13" t="str">
-        <v>../img/KhachMoi/KhongAnh.jpg</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>779292271</v>
-      </c>
-      <c r="B14" t="str">
-        <v>LÊ GIANG THÀNH</v>
-      </c>
-      <c r="C14" t="str">
-        <v>779292271</v>
-      </c>
-      <c r="D14" t="str">
-        <v>../img/KhachMoi/KhongAnh.jpg</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>777968513</v>
-      </c>
-      <c r="B15" t="str">
-        <v>NGUYỄN LÊ THANH TÚ</v>
-      </c>
-      <c r="C15" t="str">
-        <v>777968513</v>
-      </c>
-      <c r="D15" t="str">
-        <v>../img/KhachMoi/KhongAnh.jpg</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>778418962</v>
-      </c>
-      <c r="B16" t="str">
-        <v>PHẠM TẤN TRỌNG</v>
-      </c>
-      <c r="C16" t="str">
-        <v>778418962</v>
-      </c>
-      <c r="D16" t="str">
-        <v>../img/KhachMoi/KhongAnh.jpg</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>